<commit_message>
refactor(inference): flatten engine network and processors
</commit_message>
<xml_diff>
--- a/analysis/qwen3_0_6b/analysis.xlsx
+++ b/analysis/qwen3_0_6b/analysis.xlsx
@@ -1,45 +1,446 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="records" sheetId="1" r:id="rId1"/>
+    <sheet name="records" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'records'!$A$1:$AB$14</definedName>
+  </definedNames>
 </workbook>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="19" customWidth="1"/>
-    <col min="15" max="15" width="21" customWidth="1"/>
-    <col min="16" max="16" width="13" customWidth="1"/>
-    <col min="17" max="17" width="10" customWidth="1"/>
-    <col min="18" max="18" width="16" customWidth="1"/>
-    <col min="19" max="19" width="28" customWidth="1"/>
-    <col min="20" max="20" width="12" customWidth="1"/>
-    <col min="21" max="21" width="25" customWidth="1"/>
-    <col min="22" max="22" width="24" customWidth="1"/>
-    <col min="23" max="23" width="30" customWidth="1"/>
-    <col min="24" max="24" width="29" customWidth="1"/>
-    <col min="25" max="25" width="30" customWidth="1"/>
-    <col min="26" max="26" width="29" customWidth="1"/>
-    <col min="27" max="27" width="23" customWidth="1"/>
-    <col min="28" max="28" width="24" customWidth="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="29" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="29" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -358,7 +759,7 @@
         <v>2</v>
       </c>
       <c r="U3" t="n">
-        <v>87.076</v>
+        <v>87.07599999999999</v>
       </c>
       <c r="W3" t="n">
         <v>2097152</v>
@@ -637,7 +1038,7 @@
         <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>75.49</v>
+        <v>75.48999999999999</v>
       </c>
       <c r="W6" t="n">
         <v>1048576</v>
@@ -1288,7 +1689,7 @@
         <v>1</v>
       </c>
       <c r="U13" t="n">
-        <v>9.569</v>
+        <v>9.569000000000001</v>
       </c>
       <c r="W13" t="n">
         <v>4096</v>
@@ -1300,7 +1701,228 @@
         <v>1.459</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>QW-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-25T12:24:21.553717+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>qwen3-0.6b</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>c1899de289a04d12100db370d81485cdf75e47ca</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 4060 Laptop GPU</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2.14.1+cu126</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>12.6</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>bfloat16</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>512</v>
+      </c>
+      <c r="L14" t="n">
+        <v>513</v>
+      </c>
+      <c r="M14" t="n">
+        <v>16</v>
+      </c>
+      <c r="N14" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" t="n">
+        <v>5</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>qwen3_cuda::paged_decode</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>[[1,16,128],[1,2,33,16,8,128],[1,33],[1],[],[],[]]</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>1</v>
+      </c>
+      <c r="U14" t="n">
+        <v>614.2670000000001</v>
+      </c>
+      <c r="V14" t="n">
+        <v>21.429</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>2.205696105957031</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>10.81344032287598</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>2162688</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>73349120</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>QW-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-25T12:37:26.233349+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>qwen3-0.6b</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>c1899de289a04d12100db370d81485cdf75e47ca</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 4060 Laptop GPU</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2.14.1+cu126</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>12.6</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>torch.bfloat16</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>512</v>
+      </c>
+      <c r="L15" t="n">
+        <v>513</v>
+      </c>
+      <c r="M15" t="n">
+        <v>16</v>
+      </c>
+      <c r="N15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" t="n">
+        <v>5</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>aten::index</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>[[33,16,8,128],[]]</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>2</v>
+      </c>
+      <c r="U15" t="n">
+        <v>14.654</v>
+      </c>
+      <c r="V15" t="n">
+        <v>30.588</v>
+      </c>
+      <c r="W15" t="n">
+        <v>2162688</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>2.710527896881104</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>1.876991987228394</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>2162688</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>73348096</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB13"/>
+  <autoFilter ref="A1:AB14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>